<commit_message>
Fix planner QA findings
</commit_message>
<xml_diff>
--- a/Daily_Planner_QA_Test_Sheet.xlsx
+++ b/Daily_Planner_QA_Test_Sheet.xlsx
@@ -11,6 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Results" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Excel Day Details" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -463,13 +464,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="80" customWidth="1" min="2" max="2"/>
-    <col width="61" customWidth="1" min="3" max="3"/>
-    <col width="80" customWidth="1" min="4" max="4"/>
+    <col width="90" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -487,17 +486,13 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12 12:10:14</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
+          <t>2026-06-12 12:44:58</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n"/>
       <c r="B3" s="2" t="n"/>
-      <c r="C3" s="2" t="n"/>
-      <c r="D3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -510,8 +505,6 @@
           <t>Count</t>
         </is>
       </c>
-      <c r="C4" s="2" t="n"/>
-      <c r="D4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -520,10 +513,8 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>90</v>
-      </c>
-      <c r="C5" s="2" t="n"/>
-      <c r="D5" s="2" t="n"/>
+        <v>166</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -532,10 +523,8 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="C6" s="2" t="n"/>
-      <c r="D6" s="2" t="n"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -546,14 +535,10 @@
       <c r="B7" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="C7" s="2" t="n"/>
-      <c r="D7" s="2" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n"/>
       <c r="B8" s="2" t="n"/>
-      <c r="C8" s="2" t="n"/>
-      <c r="D8" s="2" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -563,17 +548,13 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Notion markdown templates, sellable Excel workbook, local Google Sheets archive reference, and Apps Script syntax/idempotency checks.</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="n"/>
-      <c r="D9" s="2" t="n"/>
+          <t>Notion markdown templates, main Excel workbook, dated Excel copy, Apps Script, and Google Sheets archive note.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n"/>
       <c r="B10" s="2" t="n"/>
-      <c r="C10" s="2" t="n"/>
-      <c r="D10" s="2" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -582,94 +563,76 @@
         </is>
       </c>
       <c r="B11" s="2" t="n"/>
-      <c r="C11" s="2" t="n"/>
-      <c r="D11" s="2" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
+      <c r="A12" s="2" t="n"/>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Monday: C3/F3 data validations present</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>Monday has no C3/F3 data validations while Tuesday-Sunday do. This also exists in v9/v10 archives, so it was pre-existing.</t>
+          <t>No warnings or failures found.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="A13" s="2" t="n"/>
+      <c r="B13" s="2" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n"/>
+      <c r="B14" s="2" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n"/>
+      <c r="B15" s="2" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n"/>
+      <c r="B16" s="2" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n"/>
+      <c r="B17" s="2" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n"/>
+      <c r="B18" s="2" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n"/>
+      <c r="B19" s="2" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n"/>
+      <c r="B20" s="2" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n"/>
+      <c r="B21" s="2" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n"/>
+      <c r="B22" s="2" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n"/>
+      <c r="B23" s="2" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
         <is>
           <t>Google Sheets archive</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>v9 archive reflects unpatched live-sheet structure</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>Old wording hits: [('How to Use', 'B21', '  2.  Schedule (6 AM – 9 PM)')]; gratitude states (has4, has5): [('Monday', True, False), ('Tuesday', True, False), ('Wednesday', True, False), ('Thursday', True, False), ('Friday', True, False), ('Saturday', True, False), ('Sunday', True, False)]. Owner still needs to run Apps Script in live Google Sheet.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>Cross-version consistency</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>No social media habit label matches across Excel and Notion</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>Excel uses "No social media 1hr" while Notion uses "No social media 1 hr". Meaning is clear, but marketplace products should use identical copy.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>Notion monthly</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>Potential 5-week month support</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>Only Week 1-4 rows are present; many months span 5 calendar weeks. Consider adding Week 5 if the product promises full-month coverage.</t>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>v9 remains an unpatched read-only archive/reference. The live Google Sheet should be fixed by running FIX_GRATITUDE_AND_WORDING_SCRIPT.txt.</t>
         </is>
       </c>
     </row>
@@ -687,14 +650,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E95"/>
+  <dimension ref="A1:E167"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="27" customWidth="1" min="1" max="1"/>
+    <col width="45" customWidth="1" min="1" max="1"/>
     <col width="61" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="80" customWidth="1" min="5" max="5"/>
+    <col width="90" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -727,7 +690,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Excel</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -750,12 +713,12 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Excel</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Sheet list matches expected structure</t>
+          <t>Expected sheets present</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
@@ -770,19 +733,19 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Found: ['How to Use', 'Monday', 'Tuesday', 'Wednesday', 'Thursday', 'Friday', 'Saturday', 'Sunday', 'Weekly Summary', 'Monthly Dashboard']</t>
+          <t>['How to Use', 'Monday', 'Tuesday', 'Wednesday', 'Thursday', 'Friday', 'Saturday', 'Sunday', 'Weekly Summary', 'Monthly Dashboard']</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Excel</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Old schedule wording removed everywhere</t>
+          <t>Old schedule wording absent</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -804,12 +767,12 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Excel</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>New schedule wording appears exactly once on How to Use</t>
+          <t>New schedule wording appears once on How to Use</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -831,12 +794,12 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Excel</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>How to Use!E1 data validation preserved</t>
+          <t>How to Use!E1 validation preserved</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -851,19 +814,19 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Data validations: ['E1']</t>
+          <t>['E1']</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Excel</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>How to Use!E1 pink-button fill preserved</t>
+          <t>How to Use!E1 pink fill preserved</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -878,19 +841,19 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Fill: FFF8C8D6</t>
+          <t>FFF8C8D6</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Excel</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>How to Use wording cell is B21</t>
+          <t>Habit label normalized to No social media 1 hr</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -900,19 +863,19 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>[('How to Use', 'B21', '  2.  Schedule (24-hour)')]</t>
+          <t>Checked all workbook text</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -928,14 +891,14 @@
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>A48:A52 = [1, 2, 3, 4, 5]</t>
+          <t>A48:A52=[1, 2, 3, 4, 5]</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -955,14 +918,14 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Row 51: 15.0; row 52: 15.0</t>
+          <t>15.0 vs 15.0</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -982,14 +945,14 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Row 51: [70, 70, 126, 126, 126, 63, 63, 63, 75, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126]; row 52: [70, 70, 126, 126, 126, 63, 63, 63, 75, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126]</t>
+          <t>Compared all columns</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -1009,14 +972,14 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Row4: [(2, 5)]; Row5: [(2, 5)]</t>
+          <t>[(2, 5)] vs [(2, 5)]</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -1036,14 +999,14 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>C3="='How to Use'!E1 - WEEKDAY('How to Use'!E1, 3)"</t>
+          <t>"='How to Use'!E1 - WEEKDAY('How to Use'!E1, 3)"</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1063,24 +1026,24 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Matches: [(7, 4, 'time-values')]</t>
+          <t>Checked 24 consecutive times</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Monday: C3/F3 data validations present</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>WARN</t>
+          <t>Monday: C3/F3 validations present</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -1090,14 +1053,14 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Monday has no C3/F3 data validations while Tuesday-Sunday do. This also exists in v9/v10 archives, so it was pre-existing.</t>
+          <t>['C3', 'F3']</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1113,14 +1076,14 @@
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>A48:A52 = [1, 2, 3, 4, 5]</t>
+          <t>A48:A52=[1, 2, 3, 4, 5]</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -1140,14 +1103,14 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Row 51: 15.0; row 52: 15.0</t>
+          <t>15.0 vs 15.0</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1167,14 +1130,14 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Row 51: [70, 70, 126, 126, 126, 63, 63, 63, 75, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126]; row 52: [70, 70, 126, 126, 126, 63, 63, 63, 75, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126]</t>
+          <t>Compared all columns</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1194,14 +1157,14 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Row4: [(2, 5)]; Row5: [(2, 5)]</t>
+          <t>[(2, 5)] vs [(2, 5)]</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1221,14 +1184,14 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>C3="='How to Use'!E1 - WEEKDAY('How to Use'!E1, 3) + 1"</t>
+          <t>"='How to Use'!E1 - WEEKDAY('How to Use'!E1, 3) + 1"</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -1248,19 +1211,19 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Matches: [(7, 4, 'time-values')]</t>
+          <t>Checked 24 consecutive times</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Tuesday: C3/F3 data validations present</t>
+          <t>Tuesday: C3/F3 validations present</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
@@ -1268,17 +1231,21 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="D22" s="2" t="inlineStr"/>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Data validations: ['C3', 'F3']</t>
+          <t>['C3', 'F3']</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -1305,7 +1272,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -1332,7 +1299,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -1359,7 +1326,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -1375,14 +1342,14 @@
       <c r="D26" s="2" t="inlineStr"/>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>A48:A52 = [1, 2, 3, 4, 5]</t>
+          <t>A48:A52=[1, 2, 3, 4, 5]</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -1402,14 +1369,14 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Row 51: 15.0; row 52: 15.0</t>
+          <t>15.0 vs 15.0</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -1429,14 +1396,14 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Row 51: [70, 70, 126, 126, 126, 63, 63, 63, 75, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126]; row 52: [70, 70, 126, 126, 126, 63, 63, 63, 75, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126]</t>
+          <t>Compared all columns</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -1456,14 +1423,14 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Row4: [(2, 5)]; Row5: [(2, 5)]</t>
+          <t>[(2, 5)] vs [(2, 5)]</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -1483,14 +1450,14 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>C3="='How to Use'!E1 - WEEKDAY('How to Use'!E1, 3) + 2"</t>
+          <t>"='How to Use'!E1 - WEEKDAY('How to Use'!E1, 3) + 2"</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -1510,19 +1477,19 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Matches: [(7, 4, 'time-values')]</t>
+          <t>Checked 24 consecutive times</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Wednesday: C3/F3 data validations present</t>
+          <t>Wednesday: C3/F3 validations present</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
@@ -1530,17 +1497,21 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="D32" s="2" t="inlineStr"/>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Data validations: ['C3', 'F3']</t>
+          <t>['C3', 'F3']</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -1567,7 +1538,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -1594,7 +1565,7 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -1621,7 +1592,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -1637,14 +1608,14 @@
       <c r="D36" s="2" t="inlineStr"/>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>A48:A52 = [1, 2, 3, 4, 5]</t>
+          <t>A48:A52=[1, 2, 3, 4, 5]</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -1664,14 +1635,14 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Row 51: 15.0; row 52: 15.0</t>
+          <t>15.0 vs 15.0</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -1691,14 +1662,14 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Row 51: [70, 70, 126, 126, 126, 63, 63, 63, 75, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126]; row 52: [70, 70, 126, 126, 126, 63, 63, 63, 75, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126]</t>
+          <t>Compared all columns</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -1718,14 +1689,14 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Row4: [(2, 5)]; Row5: [(2, 5)]</t>
+          <t>[(2, 5)] vs [(2, 5)]</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -1745,14 +1716,14 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>C3="='How to Use'!E1 - WEEKDAY('How to Use'!E1, 3) + 3"</t>
+          <t>"='How to Use'!E1 - WEEKDAY('How to Use'!E1, 3) + 3"</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
@@ -1772,19 +1743,19 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Matches: [(7, 4, 'time-values')]</t>
+          <t>Checked 24 consecutive times</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Thursday: C3/F3 data validations present</t>
+          <t>Thursday: C3/F3 validations present</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
@@ -1792,17 +1763,21 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="D42" s="2" t="inlineStr"/>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Data validations: ['C3', 'F3']</t>
+          <t>['C3', 'F3']</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
@@ -1829,7 +1804,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -1856,7 +1831,7 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
@@ -1883,7 +1858,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -1899,14 +1874,14 @@
       <c r="D46" s="2" t="inlineStr"/>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>A48:A52 = [1, 2, 3, 4, 5]</t>
+          <t>A48:A52=[1, 2, 3, 4, 5]</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
@@ -1926,14 +1901,14 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>Row 51: 15.0; row 52: 15.0</t>
+          <t>15.0 vs 15.0</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
@@ -1953,14 +1928,14 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>Row 51: [70, 70, 126, 126, 126, 63, 63, 63, 75, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126]; row 52: [70, 70, 126, 126, 126, 63, 63, 63, 75, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126]</t>
+          <t>Compared all columns</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
@@ -1980,14 +1955,14 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>Row4: [(2, 5)]; Row5: [(2, 5)]</t>
+          <t>[(2, 5)] vs [(2, 5)]</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
@@ -2007,14 +1982,14 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>C3="='How to Use'!E1 - WEEKDAY('How to Use'!E1, 3) + 4"</t>
+          <t>"='How to Use'!E1 - WEEKDAY('How to Use'!E1, 3) + 4"</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
@@ -2034,19 +2009,19 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>Matches: [(7, 4, 'time-values')]</t>
+          <t>Checked 24 consecutive times</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Friday: C3/F3 data validations present</t>
+          <t>Friday: C3/F3 validations present</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
@@ -2054,17 +2029,21 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="D52" s="2" t="inlineStr"/>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Data validations: ['C3', 'F3']</t>
+          <t>['C3', 'F3']</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
@@ -2091,7 +2070,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
@@ -2118,7 +2097,7 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
@@ -2145,7 +2124,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
@@ -2161,14 +2140,14 @@
       <c r="D56" s="2" t="inlineStr"/>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>A48:A52 = [1, 2, 3, 4, 5]</t>
+          <t>A48:A52=[1, 2, 3, 4, 5]</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
@@ -2188,14 +2167,14 @@
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>Row 51: 15.0; row 52: 15.0</t>
+          <t>15.0 vs 15.0</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
@@ -2215,14 +2194,14 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>Row 51: [70, 70, 126, 126, 126, 63, 63, 63, 75, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126]; row 52: [70, 70, 126, 126, 126, 63, 63, 63, 75, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126]</t>
+          <t>Compared all columns</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
@@ -2242,14 +2221,14 @@
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>Row4: [(2, 5)]; Row5: [(2, 5)]</t>
+          <t>[(2, 5)] vs [(2, 5)]</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
@@ -2269,14 +2248,14 @@
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>C3="='How to Use'!E1 - WEEKDAY('How to Use'!E1, 3) + 5"</t>
+          <t>"='How to Use'!E1 - WEEKDAY('How to Use'!E1, 3) + 5"</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
@@ -2296,19 +2275,19 @@
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>Matches: [(7, 4, 'time-values')]</t>
+          <t>Checked 24 consecutive times</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Saturday: C3/F3 data validations present</t>
+          <t>Saturday: C3/F3 validations present</t>
         </is>
       </c>
       <c r="C62" s="3" t="inlineStr">
@@ -2316,17 +2295,21 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="D62" s="2" t="inlineStr"/>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>Data validations: ['C3', 'F3']</t>
+          <t>['C3', 'F3']</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
@@ -2353,7 +2336,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
@@ -2380,7 +2363,7 @@
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
@@ -2407,7 +2390,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -2423,14 +2406,14 @@
       <c r="D66" s="2" t="inlineStr"/>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>A48:A52 = [1, 2, 3, 4, 5]</t>
+          <t>A48:A52=[1, 2, 3, 4, 5]</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
@@ -2450,14 +2433,14 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>Row 51: 15.0; row 52: 15.0</t>
+          <t>15.0 vs 15.0</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
@@ -2477,14 +2460,14 @@
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>Row 51: [70, 70, 126, 126, 126, 63, 63, 63, 75, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126]; row 52: [70, 70, 126, 126, 126, 63, 63, 63, 75, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126, 126]</t>
+          <t>Compared all columns</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
@@ -2504,14 +2487,14 @@
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>Row4: [(2, 5)]; Row5: [(2, 5)]</t>
+          <t>[(2, 5)] vs [(2, 5)]</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
@@ -2531,14 +2514,14 @@
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>C3="='How to Use'!E1 - WEEKDAY('How to Use'!E1, 3) + 6"</t>
+          <t>"='How to Use'!E1 - WEEKDAY('How to Use'!E1, 3) + 6"</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
@@ -2558,19 +2541,19 @@
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>Matches: [(7, 4, 'time-values')]</t>
+          <t>Checked 24 consecutive times</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>Sunday: C3/F3 data validations present</t>
+          <t>Sunday: C3/F3 validations present</t>
         </is>
       </c>
       <c r="C72" s="3" t="inlineStr">
@@ -2578,17 +2561,21 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="D72" s="2" t="inlineStr"/>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>Data validations: ['C3', 'F3']</t>
+          <t>['C3', 'F3']</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
@@ -2615,7 +2602,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
@@ -2642,7 +2629,7 @@
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>Excel day tabs</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
@@ -2669,7 +2656,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>Excel</t>
+          <t>Daily_Planner_Tracker_Excel.xlsx</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
@@ -2696,39 +2683,35 @@
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>Google Sheets archive</t>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>v9 archive reflects unpatched live-sheet structure</t>
-        </is>
-      </c>
-      <c r="C77" s="4" t="inlineStr">
-        <is>
-          <t>WARN</t>
-        </is>
-      </c>
-      <c r="D77" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
+          <t>Workbook opens</t>
+        </is>
+      </c>
+      <c r="C77" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr"/>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>Old wording hits: [('How to Use', 'B21', '  2.  Schedule (6 AM – 9 PM)')]; gratitude states (has4, has5): [('Monday', True, False), ('Tuesday', True, False), ('Wednesday', True, False), ('Thursday', True, False), ('Friday', True, False), ('Saturday', True, False), ('Sunday', True, False)]. Owner still needs to run Apps Script in live Google Sheet.</t>
+          <t>C:\Users\Charles\Documents\dwm\BloomPlansCo\Daily Planner\Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>Apps Script</t>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>Fix script exists</t>
+          <t>Expected sheets present</t>
         </is>
       </c>
       <c r="C78" s="3" t="inlineStr">
@@ -2743,19 +2726,19 @@
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>C:\Users\Charles\Documents\dwm\BloomPlansCo\Daily Planner\FIX_GRATITUDE_AND_WORDING_SCRIPT.txt</t>
+          <t>['How to Use', 'Monday', 'Tuesday', 'Wednesday', 'Thursday', 'Friday', 'Saturday', 'Sunday', 'Weekly Summary', 'Monthly Dashboard']</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>Apps Script</t>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>Function name is fixGratitudeAndWording</t>
+          <t>Old schedule wording absent</t>
         </is>
       </c>
       <c r="C79" s="3" t="inlineStr">
@@ -2768,17 +2751,21 @@
           <t>High</t>
         </is>
       </c>
-      <c r="E79" s="2" t="inlineStr"/>
+      <c r="E79" s="2" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>Apps Script</t>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>Uses insertRowsAfter and final Done alert</t>
+          <t>New schedule wording appears once on How to Use</t>
         </is>
       </c>
       <c r="C80" s="3" t="inlineStr">
@@ -2791,17 +2778,21 @@
           <t>High</t>
         </is>
       </c>
-      <c r="E80" s="2" t="inlineStr"/>
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t>[('How to Use', 'B21', '  2.  Schedule (24-hour)')]</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>Apps Script</t>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>Includes idempotency guard for existing 5 label</t>
+          <t>How to Use!E1 validation preserved</t>
         </is>
       </c>
       <c r="C81" s="3" t="inlineStr">
@@ -2814,17 +2805,21 @@
           <t>High</t>
         </is>
       </c>
-      <c r="E81" s="2" t="inlineStr"/>
+      <c r="E81" s="2" t="inlineStr">
+        <is>
+          <t>['E1']</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>Apps Script</t>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>No eval usage</t>
+          <t>How to Use!E1 pink fill preserved</t>
         </is>
       </c>
       <c r="C82" s="3" t="inlineStr">
@@ -2834,20 +2829,24 @@
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="E82" s="2" t="inlineStr"/>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="inlineStr">
+        <is>
+          <t>FFF8C8D6</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>Apps Script</t>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>Syntax parses with Node checker</t>
+          <t>Habit label normalized to No social media 1 hr</t>
         </is>
       </c>
       <c r="C83" s="3" t="inlineStr">
@@ -2857,20 +2856,24 @@
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="E83" s="2" t="inlineStr"/>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E83" s="2" t="inlineStr">
+        <is>
+          <t>Checked all workbook text</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>Notion daily</t>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>Daily markdown file exists</t>
+          <t>Monday: gratitude labels 1-5 consecutive</t>
         </is>
       </c>
       <c r="C84" s="3" t="inlineStr">
@@ -2881,19 +2884,19 @@
       <c r="D84" s="2" t="inlineStr"/>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>C:\Users\Charles\Documents\dwm\BloomPlansCo\Daily Planner\Notion_1_Daily_Page.md</t>
+          <t>A48:A52=[1, 2, 3, 4, 5]</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>Notion daily</t>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>24-hour schedule rows from 12 AM to 11 PM</t>
+          <t>Monday: row 5 height matches row 4</t>
         </is>
       </c>
       <c r="C85" s="3" t="inlineStr">
@@ -2903,24 +2906,24 @@
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>Found 24 rows: ['12:00 AM', '1:00 AM', '2:00 AM', '3:00 AM', '4:00 AM', '5:00 AM', '6:00 AM', '7:00 AM', '8:00 AM', '9:00 AM', '10:00 AM', '11:00 AM', '12:00 PM', '1:00 PM', '2:00 PM', '3:00 PM', '4:00 PM', '5:00 PM', '6:00 PM', '7:00 PM', '8:00 PM', '9:00 PM', '10:00 PM', '11:00 PM']</t>
+          <t>15.0 vs 15.0</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>Notion daily</t>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>Five gratitude entries</t>
+          <t>Monday: row 5 style IDs mirror row 4</t>
         </is>
       </c>
       <c r="C86" s="3" t="inlineStr">
@@ -2930,24 +2933,24 @@
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>Found: ['1', '2', '3', '4', '5']</t>
+          <t>Compared all columns</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>Notion daily</t>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>Top 3 priorities has exactly 3 checkboxes</t>
+          <t>Monday: row 5 merge pattern mirrors row 4</t>
         </is>
       </c>
       <c r="C87" s="3" t="inlineStr">
@@ -2957,24 +2960,24 @@
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>Checkbox count: 3</t>
+          <t>[(2, 5)] vs [(2, 5)]</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>Notion daily</t>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>To-do list has 8 checkboxes</t>
+          <t>Monday: C3 date formula unchanged</t>
         </is>
       </c>
       <c r="C88" s="3" t="inlineStr">
@@ -2984,24 +2987,24 @@
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>Checkbox count: 8</t>
+          <t>"='How to Use'!E1 - WEEKDAY('How to Use'!E1, 3)"</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>Notion daily</t>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
         </is>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>Daily goals has 5 checkboxes</t>
+          <t>Monday: 24-hour schedule present</t>
         </is>
       </c>
       <c r="C89" s="3" t="inlineStr">
@@ -3011,24 +3014,24 @@
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="E89" s="2" t="inlineStr">
         <is>
-          <t>Checkbox count: 5</t>
+          <t>Checked 24 consecutive times</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>Notion weekly</t>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>Weekly summary has Mon-Sun habit columns</t>
+          <t>Monday: C3/F3 validations present</t>
         </is>
       </c>
       <c r="C90" s="3" t="inlineStr">
@@ -3038,20 +3041,24 @@
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="E90" s="2" t="inlineStr"/>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="inlineStr">
+        <is>
+          <t>['C3', 'F3']</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>Notion weekly</t>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
         </is>
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>Weekly mood table includes average column</t>
+          <t>Tuesday: gratitude labels 1-5 consecutive</t>
         </is>
       </c>
       <c r="C91" s="3" t="inlineStr">
@@ -3059,49 +3066,49 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="D91" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E91" s="2" t="inlineStr"/>
+      <c r="D91" s="2" t="inlineStr"/>
+      <c r="E91" s="2" t="inlineStr">
+        <is>
+          <t>A48:A52=[1, 2, 3, 4, 5]</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>Cross-version consistency</t>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>No social media habit label matches across Excel and Notion</t>
-        </is>
-      </c>
-      <c r="C92" s="4" t="inlineStr">
-        <is>
-          <t>WARN</t>
+          <t>Tuesday: row 5 height matches row 4</t>
+        </is>
+      </c>
+      <c r="C92" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
         <is>
-          <t>Excel uses "No social media 1hr" while Notion uses "No social media 1 hr". Meaning is clear, but marketplace products should use identical copy.</t>
+          <t>15.0 vs 15.0</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>Notion monthly</t>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
         </is>
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>Monthly dashboard includes Week 1-4 score rows</t>
+          <t>Tuesday: row 5 style IDs mirror row 4</t>
         </is>
       </c>
       <c r="C93" s="3" t="inlineStr">
@@ -3111,24 +3118,24 @@
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E93" s="2" t="inlineStr">
         <is>
-          <t>Weeks found: ['1', '2', '3', '4']</t>
+          <t>Compared all columns</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>Notion monthly</t>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>Monthly dashboard includes monthly average row</t>
+          <t>Tuesday: row 5 merge pattern mirrors row 4</t>
         </is>
       </c>
       <c r="C94" s="3" t="inlineStr">
@@ -3141,34 +3148,1922 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="E94" s="2" t="inlineStr"/>
+      <c r="E94" s="2" t="inlineStr">
+        <is>
+          <t>[(2, 5)] vs [(2, 5)]</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
+        </is>
+      </c>
+      <c r="B95" s="2" t="inlineStr">
+        <is>
+          <t>Tuesday: C3 date formula unchanged</t>
+        </is>
+      </c>
+      <c r="C95" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D95" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E95" s="2" t="inlineStr">
+        <is>
+          <t>"='How to Use'!E1 - WEEKDAY('How to Use'!E1, 3) + 1"</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>Tuesday: 24-hour schedule present</t>
+        </is>
+      </c>
+      <c r="C96" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E96" s="2" t="inlineStr">
+        <is>
+          <t>Checked 24 consecutive times</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
+        </is>
+      </c>
+      <c r="B97" s="2" t="inlineStr">
+        <is>
+          <t>Tuesday: C3/F3 validations present</t>
+        </is>
+      </c>
+      <c r="C97" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D97" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E97" s="2" t="inlineStr">
+        <is>
+          <t>['C3', 'F3']</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
+        </is>
+      </c>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t>Tuesday: column widths match Monday</t>
+        </is>
+      </c>
+      <c r="C98" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E98" s="2" t="inlineStr">
+        <is>
+          <t>Compared all columns</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="inlineStr">
+        <is>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
+        </is>
+      </c>
+      <c r="B99" s="2" t="inlineStr">
+        <is>
+          <t>Tuesday: merge ranges match Monday</t>
+        </is>
+      </c>
+      <c r="C99" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D99" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E99" s="2" t="inlineStr">
+        <is>
+          <t>Compared all merged ranges</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
+        </is>
+      </c>
+      <c r="B100" s="2" t="inlineStr">
+        <is>
+          <t>Tuesday: sampled row heights match Monday</t>
+        </is>
+      </c>
+      <c r="C100" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D100" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E100" s="2" t="inlineStr">
+        <is>
+          <t>Compared rows 1-80</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="inlineStr">
+        <is>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
+        </is>
+      </c>
+      <c r="B101" s="2" t="inlineStr">
+        <is>
+          <t>Wednesday: gratitude labels 1-5 consecutive</t>
+        </is>
+      </c>
+      <c r="C101" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D101" s="2" t="inlineStr"/>
+      <c r="E101" s="2" t="inlineStr">
+        <is>
+          <t>A48:A52=[1, 2, 3, 4, 5]</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="inlineStr">
+        <is>
+          <t>Wednesday: row 5 height matches row 4</t>
+        </is>
+      </c>
+      <c r="C102" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D102" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E102" s="2" t="inlineStr">
+        <is>
+          <t>15.0 vs 15.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="inlineStr">
+        <is>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
+        </is>
+      </c>
+      <c r="B103" s="2" t="inlineStr">
+        <is>
+          <t>Wednesday: row 5 style IDs mirror row 4</t>
+        </is>
+      </c>
+      <c r="C103" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D103" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E103" s="2" t="inlineStr">
+        <is>
+          <t>Compared all columns</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
+        </is>
+      </c>
+      <c r="B104" s="2" t="inlineStr">
+        <is>
+          <t>Wednesday: row 5 merge pattern mirrors row 4</t>
+        </is>
+      </c>
+      <c r="C104" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D104" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E104" s="2" t="inlineStr">
+        <is>
+          <t>[(2, 5)] vs [(2, 5)]</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="2" t="inlineStr">
+        <is>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
+        </is>
+      </c>
+      <c r="B105" s="2" t="inlineStr">
+        <is>
+          <t>Wednesday: C3 date formula unchanged</t>
+        </is>
+      </c>
+      <c r="C105" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D105" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E105" s="2" t="inlineStr">
+        <is>
+          <t>"='How to Use'!E1 - WEEKDAY('How to Use'!E1, 3) + 2"</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
+        </is>
+      </c>
+      <c r="B106" s="2" t="inlineStr">
+        <is>
+          <t>Wednesday: 24-hour schedule present</t>
+        </is>
+      </c>
+      <c r="C106" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D106" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E106" s="2" t="inlineStr">
+        <is>
+          <t>Checked 24 consecutive times</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="inlineStr">
+        <is>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
+        </is>
+      </c>
+      <c r="B107" s="2" t="inlineStr">
+        <is>
+          <t>Wednesday: C3/F3 validations present</t>
+        </is>
+      </c>
+      <c r="C107" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D107" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E107" s="2" t="inlineStr">
+        <is>
+          <t>['C3', 'F3']</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="inlineStr">
+        <is>
+          <t>Wednesday: column widths match Monday</t>
+        </is>
+      </c>
+      <c r="C108" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D108" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E108" s="2" t="inlineStr">
+        <is>
+          <t>Compared all columns</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="inlineStr">
+        <is>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
+        </is>
+      </c>
+      <c r="B109" s="2" t="inlineStr">
+        <is>
+          <t>Wednesday: merge ranges match Monday</t>
+        </is>
+      </c>
+      <c r="C109" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D109" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E109" s="2" t="inlineStr">
+        <is>
+          <t>Compared all merged ranges</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
+        </is>
+      </c>
+      <c r="B110" s="2" t="inlineStr">
+        <is>
+          <t>Wednesday: sampled row heights match Monday</t>
+        </is>
+      </c>
+      <c r="C110" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D110" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E110" s="2" t="inlineStr">
+        <is>
+          <t>Compared rows 1-80</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="inlineStr">
+        <is>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
+        </is>
+      </c>
+      <c r="B111" s="2" t="inlineStr">
+        <is>
+          <t>Thursday: gratitude labels 1-5 consecutive</t>
+        </is>
+      </c>
+      <c r="C111" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D111" s="2" t="inlineStr"/>
+      <c r="E111" s="2" t="inlineStr">
+        <is>
+          <t>A48:A52=[1, 2, 3, 4, 5]</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
+        </is>
+      </c>
+      <c r="B112" s="2" t="inlineStr">
+        <is>
+          <t>Thursday: row 5 height matches row 4</t>
+        </is>
+      </c>
+      <c r="C112" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D112" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E112" s="2" t="inlineStr">
+        <is>
+          <t>15.0 vs 15.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="2" t="inlineStr">
+        <is>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
+        </is>
+      </c>
+      <c r="B113" s="2" t="inlineStr">
+        <is>
+          <t>Thursday: row 5 style IDs mirror row 4</t>
+        </is>
+      </c>
+      <c r="C113" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D113" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E113" s="2" t="inlineStr">
+        <is>
+          <t>Compared all columns</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="inlineStr">
+        <is>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
+        </is>
+      </c>
+      <c r="B114" s="2" t="inlineStr">
+        <is>
+          <t>Thursday: row 5 merge pattern mirrors row 4</t>
+        </is>
+      </c>
+      <c r="C114" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D114" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E114" s="2" t="inlineStr">
+        <is>
+          <t>[(2, 5)] vs [(2, 5)]</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="2" t="inlineStr">
+        <is>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
+        </is>
+      </c>
+      <c r="B115" s="2" t="inlineStr">
+        <is>
+          <t>Thursday: C3 date formula unchanged</t>
+        </is>
+      </c>
+      <c r="C115" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D115" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E115" s="2" t="inlineStr">
+        <is>
+          <t>"='How to Use'!E1 - WEEKDAY('How to Use'!E1, 3) + 3"</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="inlineStr">
+        <is>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
+        </is>
+      </c>
+      <c r="B116" s="2" t="inlineStr">
+        <is>
+          <t>Thursday: 24-hour schedule present</t>
+        </is>
+      </c>
+      <c r="C116" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D116" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E116" s="2" t="inlineStr">
+        <is>
+          <t>Checked 24 consecutive times</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="2" t="inlineStr">
+        <is>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
+        </is>
+      </c>
+      <c r="B117" s="2" t="inlineStr">
+        <is>
+          <t>Thursday: C3/F3 validations present</t>
+        </is>
+      </c>
+      <c r="C117" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D117" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E117" s="2" t="inlineStr">
+        <is>
+          <t>['C3', 'F3']</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="2" t="inlineStr">
+        <is>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
+        </is>
+      </c>
+      <c r="B118" s="2" t="inlineStr">
+        <is>
+          <t>Thursday: column widths match Monday</t>
+        </is>
+      </c>
+      <c r="C118" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D118" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E118" s="2" t="inlineStr">
+        <is>
+          <t>Compared all columns</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="2" t="inlineStr">
+        <is>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
+        </is>
+      </c>
+      <c r="B119" s="2" t="inlineStr">
+        <is>
+          <t>Thursday: merge ranges match Monday</t>
+        </is>
+      </c>
+      <c r="C119" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D119" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E119" s="2" t="inlineStr">
+        <is>
+          <t>Compared all merged ranges</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="2" t="inlineStr">
+        <is>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
+        </is>
+      </c>
+      <c r="B120" s="2" t="inlineStr">
+        <is>
+          <t>Thursday: sampled row heights match Monday</t>
+        </is>
+      </c>
+      <c r="C120" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D120" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E120" s="2" t="inlineStr">
+        <is>
+          <t>Compared rows 1-80</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="2" t="inlineStr">
+        <is>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
+        </is>
+      </c>
+      <c r="B121" s="2" t="inlineStr">
+        <is>
+          <t>Friday: gratitude labels 1-5 consecutive</t>
+        </is>
+      </c>
+      <c r="C121" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D121" s="2" t="inlineStr"/>
+      <c r="E121" s="2" t="inlineStr">
+        <is>
+          <t>A48:A52=[1, 2, 3, 4, 5]</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
+        </is>
+      </c>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>Friday: row 5 height matches row 4</t>
+        </is>
+      </c>
+      <c r="C122" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D122" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E122" s="2" t="inlineStr">
+        <is>
+          <t>15.0 vs 15.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="2" t="inlineStr">
+        <is>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
+        </is>
+      </c>
+      <c r="B123" s="2" t="inlineStr">
+        <is>
+          <t>Friday: row 5 style IDs mirror row 4</t>
+        </is>
+      </c>
+      <c r="C123" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D123" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E123" s="2" t="inlineStr">
+        <is>
+          <t>Compared all columns</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="2" t="inlineStr">
+        <is>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
+        </is>
+      </c>
+      <c r="B124" s="2" t="inlineStr">
+        <is>
+          <t>Friday: row 5 merge pattern mirrors row 4</t>
+        </is>
+      </c>
+      <c r="C124" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D124" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E124" s="2" t="inlineStr">
+        <is>
+          <t>[(2, 5)] vs [(2, 5)]</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="2" t="inlineStr">
+        <is>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
+        </is>
+      </c>
+      <c r="B125" s="2" t="inlineStr">
+        <is>
+          <t>Friday: C3 date formula unchanged</t>
+        </is>
+      </c>
+      <c r="C125" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D125" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E125" s="2" t="inlineStr">
+        <is>
+          <t>"='How to Use'!E1 - WEEKDAY('How to Use'!E1, 3) + 4"</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="2" t="inlineStr">
+        <is>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
+        </is>
+      </c>
+      <c r="B126" s="2" t="inlineStr">
+        <is>
+          <t>Friday: 24-hour schedule present</t>
+        </is>
+      </c>
+      <c r="C126" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D126" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E126" s="2" t="inlineStr">
+        <is>
+          <t>Checked 24 consecutive times</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="2" t="inlineStr">
+        <is>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
+        </is>
+      </c>
+      <c r="B127" s="2" t="inlineStr">
+        <is>
+          <t>Friday: C3/F3 validations present</t>
+        </is>
+      </c>
+      <c r="C127" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D127" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E127" s="2" t="inlineStr">
+        <is>
+          <t>['C3', 'F3']</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="2" t="inlineStr">
+        <is>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
+        </is>
+      </c>
+      <c r="B128" s="2" t="inlineStr">
+        <is>
+          <t>Friday: column widths match Monday</t>
+        </is>
+      </c>
+      <c r="C128" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D128" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E128" s="2" t="inlineStr">
+        <is>
+          <t>Compared all columns</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="2" t="inlineStr">
+        <is>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
+        </is>
+      </c>
+      <c r="B129" s="2" t="inlineStr">
+        <is>
+          <t>Friday: merge ranges match Monday</t>
+        </is>
+      </c>
+      <c r="C129" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D129" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E129" s="2" t="inlineStr">
+        <is>
+          <t>Compared all merged ranges</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="2" t="inlineStr">
+        <is>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
+        </is>
+      </c>
+      <c r="B130" s="2" t="inlineStr">
+        <is>
+          <t>Friday: sampled row heights match Monday</t>
+        </is>
+      </c>
+      <c r="C130" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D130" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E130" s="2" t="inlineStr">
+        <is>
+          <t>Compared rows 1-80</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="2" t="inlineStr">
+        <is>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
+        </is>
+      </c>
+      <c r="B131" s="2" t="inlineStr">
+        <is>
+          <t>Saturday: gratitude labels 1-5 consecutive</t>
+        </is>
+      </c>
+      <c r="C131" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D131" s="2" t="inlineStr"/>
+      <c r="E131" s="2" t="inlineStr">
+        <is>
+          <t>A48:A52=[1, 2, 3, 4, 5]</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="2" t="inlineStr">
+        <is>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
+        </is>
+      </c>
+      <c r="B132" s="2" t="inlineStr">
+        <is>
+          <t>Saturday: row 5 height matches row 4</t>
+        </is>
+      </c>
+      <c r="C132" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D132" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E132" s="2" t="inlineStr">
+        <is>
+          <t>15.0 vs 15.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="2" t="inlineStr">
+        <is>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
+        </is>
+      </c>
+      <c r="B133" s="2" t="inlineStr">
+        <is>
+          <t>Saturday: row 5 style IDs mirror row 4</t>
+        </is>
+      </c>
+      <c r="C133" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D133" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E133" s="2" t="inlineStr">
+        <is>
+          <t>Compared all columns</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="2" t="inlineStr">
+        <is>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
+        </is>
+      </c>
+      <c r="B134" s="2" t="inlineStr">
+        <is>
+          <t>Saturday: row 5 merge pattern mirrors row 4</t>
+        </is>
+      </c>
+      <c r="C134" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D134" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E134" s="2" t="inlineStr">
+        <is>
+          <t>[(2, 5)] vs [(2, 5)]</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="2" t="inlineStr">
+        <is>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
+        </is>
+      </c>
+      <c r="B135" s="2" t="inlineStr">
+        <is>
+          <t>Saturday: C3 date formula unchanged</t>
+        </is>
+      </c>
+      <c r="C135" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D135" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E135" s="2" t="inlineStr">
+        <is>
+          <t>"='How to Use'!E1 - WEEKDAY('How to Use'!E1, 3) + 5"</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="2" t="inlineStr">
+        <is>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
+        </is>
+      </c>
+      <c r="B136" s="2" t="inlineStr">
+        <is>
+          <t>Saturday: 24-hour schedule present</t>
+        </is>
+      </c>
+      <c r="C136" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D136" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E136" s="2" t="inlineStr">
+        <is>
+          <t>Checked 24 consecutive times</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="2" t="inlineStr">
+        <is>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
+        </is>
+      </c>
+      <c r="B137" s="2" t="inlineStr">
+        <is>
+          <t>Saturday: C3/F3 validations present</t>
+        </is>
+      </c>
+      <c r="C137" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D137" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E137" s="2" t="inlineStr">
+        <is>
+          <t>['C3', 'F3']</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="2" t="inlineStr">
+        <is>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
+        </is>
+      </c>
+      <c r="B138" s="2" t="inlineStr">
+        <is>
+          <t>Saturday: column widths match Monday</t>
+        </is>
+      </c>
+      <c r="C138" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D138" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E138" s="2" t="inlineStr">
+        <is>
+          <t>Compared all columns</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="2" t="inlineStr">
+        <is>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
+        </is>
+      </c>
+      <c r="B139" s="2" t="inlineStr">
+        <is>
+          <t>Saturday: merge ranges match Monday</t>
+        </is>
+      </c>
+      <c r="C139" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D139" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E139" s="2" t="inlineStr">
+        <is>
+          <t>Compared all merged ranges</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="2" t="inlineStr">
+        <is>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
+        </is>
+      </c>
+      <c r="B140" s="2" t="inlineStr">
+        <is>
+          <t>Saturday: sampled row heights match Monday</t>
+        </is>
+      </c>
+      <c r="C140" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D140" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E140" s="2" t="inlineStr">
+        <is>
+          <t>Compared rows 1-80</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="2" t="inlineStr">
+        <is>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
+        </is>
+      </c>
+      <c r="B141" s="2" t="inlineStr">
+        <is>
+          <t>Sunday: gratitude labels 1-5 consecutive</t>
+        </is>
+      </c>
+      <c r="C141" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D141" s="2" t="inlineStr"/>
+      <c r="E141" s="2" t="inlineStr">
+        <is>
+          <t>A48:A52=[1, 2, 3, 4, 5]</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="2" t="inlineStr">
+        <is>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
+        </is>
+      </c>
+      <c r="B142" s="2" t="inlineStr">
+        <is>
+          <t>Sunday: row 5 height matches row 4</t>
+        </is>
+      </c>
+      <c r="C142" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D142" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E142" s="2" t="inlineStr">
+        <is>
+          <t>15.0 vs 15.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="2" t="inlineStr">
+        <is>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
+        </is>
+      </c>
+      <c r="B143" s="2" t="inlineStr">
+        <is>
+          <t>Sunday: row 5 style IDs mirror row 4</t>
+        </is>
+      </c>
+      <c r="C143" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D143" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E143" s="2" t="inlineStr">
+        <is>
+          <t>Compared all columns</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="2" t="inlineStr">
+        <is>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
+        </is>
+      </c>
+      <c r="B144" s="2" t="inlineStr">
+        <is>
+          <t>Sunday: row 5 merge pattern mirrors row 4</t>
+        </is>
+      </c>
+      <c r="C144" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D144" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E144" s="2" t="inlineStr">
+        <is>
+          <t>[(2, 5)] vs [(2, 5)]</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="2" t="inlineStr">
+        <is>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
+        </is>
+      </c>
+      <c r="B145" s="2" t="inlineStr">
+        <is>
+          <t>Sunday: C3 date formula unchanged</t>
+        </is>
+      </c>
+      <c r="C145" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D145" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E145" s="2" t="inlineStr">
+        <is>
+          <t>"='How to Use'!E1 - WEEKDAY('How to Use'!E1, 3) + 6"</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="2" t="inlineStr">
+        <is>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
+        </is>
+      </c>
+      <c r="B146" s="2" t="inlineStr">
+        <is>
+          <t>Sunday: 24-hour schedule present</t>
+        </is>
+      </c>
+      <c r="C146" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D146" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E146" s="2" t="inlineStr">
+        <is>
+          <t>Checked 24 consecutive times</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="2" t="inlineStr">
+        <is>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
+        </is>
+      </c>
+      <c r="B147" s="2" t="inlineStr">
+        <is>
+          <t>Sunday: C3/F3 validations present</t>
+        </is>
+      </c>
+      <c r="C147" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D147" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E147" s="2" t="inlineStr">
+        <is>
+          <t>['C3', 'F3']</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="2" t="inlineStr">
+        <is>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
+        </is>
+      </c>
+      <c r="B148" s="2" t="inlineStr">
+        <is>
+          <t>Sunday: column widths match Monday</t>
+        </is>
+      </c>
+      <c r="C148" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D148" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E148" s="2" t="inlineStr">
+        <is>
+          <t>Compared all columns</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="2" t="inlineStr">
+        <is>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
+        </is>
+      </c>
+      <c r="B149" s="2" t="inlineStr">
+        <is>
+          <t>Sunday: merge ranges match Monday</t>
+        </is>
+      </c>
+      <c r="C149" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D149" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E149" s="2" t="inlineStr">
+        <is>
+          <t>Compared all merged ranges</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="2" t="inlineStr">
+        <is>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
+        </is>
+      </c>
+      <c r="B150" s="2" t="inlineStr">
+        <is>
+          <t>Sunday: sampled row heights match Monday</t>
+        </is>
+      </c>
+      <c r="C150" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D150" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E150" s="2" t="inlineStr">
+        <is>
+          <t>Compared rows 1-80</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="2" t="inlineStr">
+        <is>
+          <t>Daily_Planner_Tracker_Excel_2026-06-12.xlsx</t>
+        </is>
+      </c>
+      <c r="B151" s="2" t="inlineStr">
+        <is>
+          <t>No literal formula error markers found</t>
+        </is>
+      </c>
+      <c r="C151" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D151" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E151" s="2" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="2" t="inlineStr">
+        <is>
+          <t>Notion daily</t>
+        </is>
+      </c>
+      <c r="B152" s="2" t="inlineStr">
+        <is>
+          <t>24-hour schedule rows from 12 AM to 11 PM</t>
+        </is>
+      </c>
+      <c r="C152" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D152" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E152" s="2" t="inlineStr">
+        <is>
+          <t>24 rows</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="2" t="inlineStr">
+        <is>
+          <t>Notion daily</t>
+        </is>
+      </c>
+      <c r="B153" s="2" t="inlineStr">
+        <is>
+          <t>Five gratitude entries</t>
+        </is>
+      </c>
+      <c r="C153" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D153" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E153" s="2" t="inlineStr">
+        <is>
+          <t>['1', '2', '3', '4', '5']</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="2" t="inlineStr">
+        <is>
+          <t>Notion daily</t>
+        </is>
+      </c>
+      <c r="B154" s="2" t="inlineStr">
+        <is>
+          <t>Top 3 priorities has 3 checkboxes</t>
+        </is>
+      </c>
+      <c r="C154" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D154" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E154" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="2" t="inlineStr">
+        <is>
+          <t>Notion daily</t>
+        </is>
+      </c>
+      <c r="B155" s="2" t="inlineStr">
+        <is>
+          <t>To-do list has 8 checkboxes</t>
+        </is>
+      </c>
+      <c r="C155" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D155" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E155" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="2" t="inlineStr">
+        <is>
+          <t>Notion daily</t>
+        </is>
+      </c>
+      <c r="B156" s="2" t="inlineStr">
+        <is>
+          <t>Daily goals has 5 checkboxes</t>
+        </is>
+      </c>
+      <c r="C156" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D156" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E156" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="2" t="inlineStr">
+        <is>
+          <t>Notion weekly</t>
+        </is>
+      </c>
+      <c r="B157" s="2" t="inlineStr">
+        <is>
+          <t>Weekly summary has Mon-Sun habit columns</t>
+        </is>
+      </c>
+      <c r="C157" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D157" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E157" s="2" t="inlineStr"/>
+    </row>
+    <row r="158">
+      <c r="A158" s="2" t="inlineStr">
+        <is>
+          <t>Notion weekly</t>
+        </is>
+      </c>
+      <c r="B158" s="2" t="inlineStr">
+        <is>
+          <t>Weekly mood table includes average column</t>
+        </is>
+      </c>
+      <c r="C158" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D158" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E158" s="2" t="inlineStr"/>
+    </row>
+    <row r="159">
+      <c r="A159" s="2" t="inlineStr">
+        <is>
+          <t>Cross-version consistency</t>
+        </is>
+      </c>
+      <c r="B159" s="2" t="inlineStr">
+        <is>
+          <t>No social media habit label matches across Excel and Notion</t>
+        </is>
+      </c>
+      <c r="C159" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D159" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E159" s="2" t="inlineStr"/>
+    </row>
+    <row r="160">
+      <c r="A160" s="2" t="inlineStr">
+        <is>
           <t>Notion monthly</t>
         </is>
       </c>
-      <c r="B95" s="2" t="inlineStr">
-        <is>
-          <t>Potential 5-week month support</t>
-        </is>
-      </c>
-      <c r="C95" s="4" t="inlineStr">
-        <is>
-          <t>WARN</t>
-        </is>
-      </c>
-      <c r="D95" s="2" t="inlineStr">
+      <c r="B160" s="2" t="inlineStr">
+        <is>
+          <t>Monthly dashboard includes Week 1-5 score rows</t>
+        </is>
+      </c>
+      <c r="C160" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D160" s="2" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="E95" s="2" t="inlineStr">
-        <is>
-          <t>Only Week 1-4 rows are present; many months span 5 calendar weeks. Consider adding Week 5 if the product promises full-month coverage.</t>
-        </is>
-      </c>
+      <c r="E160" s="2" t="inlineStr">
+        <is>
+          <t>['1', '2', '3', '4', '5']</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="2" t="inlineStr">
+        <is>
+          <t>Notion monthly</t>
+        </is>
+      </c>
+      <c r="B161" s="2" t="inlineStr">
+        <is>
+          <t>Monthly average row present</t>
+        </is>
+      </c>
+      <c r="C161" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D161" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E161" s="2" t="inlineStr"/>
+    </row>
+    <row r="162">
+      <c r="A162" s="2" t="inlineStr">
+        <is>
+          <t>Apps Script</t>
+        </is>
+      </c>
+      <c r="B162" s="2" t="inlineStr">
+        <is>
+          <t>Fix script exists</t>
+        </is>
+      </c>
+      <c r="C162" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D162" s="2" t="inlineStr"/>
+      <c r="E162" s="2" t="inlineStr">
+        <is>
+          <t>C:\Users\Charles\Documents\dwm\BloomPlansCo\Daily Planner\FIX_GRATITUDE_AND_WORDING_SCRIPT.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="2" t="inlineStr">
+        <is>
+          <t>Apps Script</t>
+        </is>
+      </c>
+      <c r="B163" s="2" t="inlineStr">
+        <is>
+          <t>Function name is fixGratitudeAndWording</t>
+        </is>
+      </c>
+      <c r="C163" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D163" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E163" s="2" t="inlineStr"/>
+    </row>
+    <row r="164">
+      <c r="A164" s="2" t="inlineStr">
+        <is>
+          <t>Apps Script</t>
+        </is>
+      </c>
+      <c r="B164" s="2" t="inlineStr">
+        <is>
+          <t>Uses insertRowsAfter and Done alert</t>
+        </is>
+      </c>
+      <c r="C164" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D164" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E164" s="2" t="inlineStr"/>
+    </row>
+    <row r="165">
+      <c r="A165" s="2" t="inlineStr">
+        <is>
+          <t>Apps Script</t>
+        </is>
+      </c>
+      <c r="B165" s="2" t="inlineStr">
+        <is>
+          <t>Includes idempotency guard</t>
+        </is>
+      </c>
+      <c r="C165" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D165" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E165" s="2" t="inlineStr"/>
+    </row>
+    <row r="166">
+      <c r="A166" s="2" t="inlineStr">
+        <is>
+          <t>Apps Script</t>
+        </is>
+      </c>
+      <c r="B166" s="2" t="inlineStr">
+        <is>
+          <t>No eval usage</t>
+        </is>
+      </c>
+      <c r="C166" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D166" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E166" s="2" t="inlineStr"/>
+    </row>
+    <row r="167">
+      <c r="A167" s="2" t="inlineStr">
+        <is>
+          <t>Apps Script</t>
+        </is>
+      </c>
+      <c r="B167" s="2" t="inlineStr">
+        <is>
+          <t>Syntax parses with Node checker</t>
+        </is>
+      </c>
+      <c r="C167" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D167" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E167" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3181,13 +5076,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="27" customWidth="1" min="2" max="2"/>
-    <col width="61" customWidth="1" min="3" max="3"/>
-    <col width="80" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3209,94 +5104,6 @@
       <c r="D1" s="6" t="inlineStr">
         <is>
           <t>Details</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Excel day tabs</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Monday: C3/F3 data validations present</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Monday has no C3/F3 data validations while Tuesday-Sunday do. This also exists in v9/v10 archives, so it was pre-existing.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Google Sheets archive</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>v9 archive reflects unpatched live-sheet structure</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Old wording hits: [('How to Use', 'B21', '  2.  Schedule (6 AM – 9 PM)')]; gratitude states (has4, has5): [('Monday', True, False), ('Tuesday', True, False), ('Wednesday', True, False), ('Thursday', True, False), ('Friday', True, False), ('Saturday', True, False), ('Sunday', True, False)]. Owner still needs to run Apps Script in live Google Sheet.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Cross-version consistency</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>No social media habit label matches across Excel and Notion</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Excel uses "No social media 1hr" while Notion uses "No social media 1 hr". Meaning is clear, but marketplace products should use identical copy.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Notion monthly</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Potential 5-week month support</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Only Week 1-4 rows are present; many months span 5 calendar weeks. Consider adding Week 5 if the product promises full-month coverage.</t>
         </is>
       </c>
     </row>
@@ -3366,7 +5173,11 @@
         <f>'How to Use'!E1 - WEEKDAY('How to Use'!E1, 3)</f>
         <v/>
       </c>
-      <c r="E2" s="2" t="inlineStr"/>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>C3, F3</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -3509,6 +5320,48 @@
       <c r="E8" s="2" t="inlineStr">
         <is>
           <t>C3, F3</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="23" customWidth="1" min="1" max="1"/>
+    <col width="90" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Area</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Google Sheets archive</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>v9 remains an unpatched read-only archive/reference. The live Google Sheet should be fixed by running FIX_GRATITUDE_AND_WORDING_SCRIPT.txt.</t>
         </is>
       </c>
     </row>

</xml_diff>